<commit_message>
HU-046 v1 ajuste: valor Allocated no SerializedProduct.Status (par com Available), modelo de 2 campos da HU preservado
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk1sLCwJ9hwDtqy7bSFwgQ
</commit_message>
<xml_diff>
--- a/docs/HU046_Tarefas_Tecnicas_v1.xlsx
+++ b/docs/HU046_Tarefas_Tecnicas_v1.xlsx
@@ -199,7 +199,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">"En demostracion" YA existe (describe 05/08; "En consignacion" tambien). Agregar 2 valores con label ES. NO se crea campo: Vehicle.Status es la FUENTE UNICA del bloqueo comercial (ver D1 - SerializedProduct.Status no tiene semantica de asignacion y se queda con su ciclo de stock)</t>
+          <t xml:space="preserve">"En demostracion" YA existe (describe 05/08; "En consignacion" tambien). Agregar: Vehicle.Status "En exhibicion" + "Demo venta" Y SerializedProduct.Status "Allocated" (label ES "Asignado") - valor de picklist standard, NO campo custom. "Deallocated" NO se crea: el retorno es "Available", que ya existe. VERIFICAR 1-click que SerializedProduct.Status acepta valores nuevos (Object Manager). Modelo de 2 campos de la HU preservado: Status del SerializedProduct = disponibilidad; Vehicle.Status = uso</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">No existe SerializedProduct.AllocationStatus ni el valor Allocated (describe 05/08: Status = Available/Sent/Consumed/Damaged/Lost). El bloqueo real es Vehicle.Status como fuente unica + guarda en QuoteOrderService. "Sale de QuantityAvailable" tampoco esta verificado: la cantidad sigue con SAP maestro + filtros del flujo. Ajustar la redaccion de la HU con Meli ANTES de que QA pruebe contra un campo inexistente</t>
+          <t xml:space="preserve">No existe el campo SerializedProduct.AllocationStatus (describe 05/08): el campo real es SerializedProduct.Status (Available/Sent/Consumed/Damaged/Lost). SOLUCION RECOMENDADA: agregar el valor "Allocated" al picklist standard (T03) - preserva el modelo de 2 campos de la HU con 1 valor nuevo; "Deallocated" = "Available" (ya existe). Guarda comercial en QuoteOrderService complementa. "Sale de QuantityAvailable" NO verificado: la cantidad sigue con SAP maestro + filtros. Ajustar redaccion de la HU con Meli (nombre del campo + par Allocated/Available) ANTES de QA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle.Status (fuente unica: En demostracion / En exhibicion) + guarda en QuoteOrderService</t>
+          <t xml:space="preserve">SerializedProduct.Status = Allocated (disponibilidad) + Vehicle.Status = En demostracion / En exhibicion (uso) + guarda en QuoteOrderService</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HU-046 v1: T01/T02 atualizadas - CBSF ativo com configuracoes existentes na org (reaproveitar Grupo Q Busqueda de Vehiculos)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk1sLCwJ9hwDtqy7bSFwgQ
</commit_message>
<xml_diff>
--- a/docs/HU046_Tarefas_Tecnicas_v1.xlsx
+++ b/docs/HU046_Tarefas_Tecnicas_v1.xlsx
@@ -125,7 +125,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configurar Criteria-Based Search and Filter sobre el objeto Vehicle DIRECTO (sin Data Processing Engine en R1 - doc oficial: con Vehicle no se requiere DPE). Definir campos de filtro (marca, modelo, ubicacion, VIN, color, estado), resultado, orden y agregacion. Agregar el componente CBSF a la app GrupoQ Ventas. VERIFICAR el nodo de Setup (Quick Find "Criteria") o los tipos de metadata via Inspector - Automotive base Active confirmado 05/08; VehicleSearchableField existe en la org</t>
+          <t xml:space="preserve">CBSF Active en la org (verificado 05/08) y YA EXISTEN 3 Search Configurations: "Grupo Q Busqueda de Vehiculos" (ACTIVE, sobre Vehicle), "Search Vehicle Inventory" (inactive) y "Buscar producto" (DealerProdtSearchableField, inactive). Tarea = AUDITAR/EXTENDER la configuracion activa para el escenario demo (filtros de estado/ubicacion, columnas, agregacion), definir con el equipo cual de las 2 de Vehicle queda como oficial (desactivar la otra), y exponer el componente CBSF a gerentes/encargados. Sin DPE (Vehicle directo)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -162,7 +162,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accion LWC Vehicle Transfer ENTREGADA por el producto: seleccion multiple de resultados y traslado a la ubicacion destino (CDA -&gt; sala). Movimiento via ProductTransfer con log automatico en SerializedProductTransaction (valores Received/Sent/Adjusted... confirmados 05/08)</t>
+          <t xml:space="preserve">Accion LWC Vehicle Transfer ENTREGADA por el producto: seleccion multiple de resultados y traslado a la ubicacion destino (CDA -&gt; sala). Revisar la pestana Action Configuration del Setup CBSF (existe en la org) y sumar la accion a la configuracion oficial. Movimiento via ProductTransfer con log automatico en SerializedProductTransaction (valores confirmados 05/08)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">

</xml_diff>